<commit_message>
Demo file per language, two classification routes, cross-source checks
- An English and a French demo file (French headers, semicolons, decimal
  commas); the import screen offers the one matching the language.
- Classification: Altera reference base, then the language model; non-food
  shown as out of scope. No unanimous segment.
- Quality checks: consistency between sources for protein values and the
  NEVO split.
- Deliverables take about 20 seconds, the insights report first.
- Top bar: Altera.ai, then DEMO.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/downloads/HarbourMarket_Protein_Ratio_DEMO.xlsx
+++ b/public/downloads/HarbourMarket_Protein_Ratio_DEMO.xlsx
@@ -3600,7 +3600,7 @@
       </c>
       <c r="P7" s="15" t="inlineStr">
         <is>
-          <t>Unanimous segment</t>
+          <t>Altera reference base</t>
         </is>
       </c>
       <c r="Q7" s="42" t="n"/>
@@ -4138,10 +4138,12 @@
       </c>
       <c r="P11" s="15" t="inlineStr">
         <is>
-          <t>Unanimous segment</t>
-        </is>
-      </c>
-      <c r="Q11" s="42" t="n"/>
+          <t>Language model</t>
+        </is>
+      </c>
+      <c r="Q11" s="42" t="n">
+        <v>0.97</v>
+      </c>
       <c r="R11" s="43" t="n">
         <v>118000</v>
       </c>
@@ -4272,7 +4274,7 @@
       </c>
       <c r="P12" s="15" t="inlineStr">
         <is>
-          <t>Unanimous segment</t>
+          <t>Altera reference base</t>
         </is>
       </c>
       <c r="Q12" s="42" t="n"/>
@@ -4674,7 +4676,7 @@
       </c>
       <c r="P15" s="15" t="inlineStr">
         <is>
-          <t>Unanimous segment</t>
+          <t>Altera reference base</t>
         </is>
       </c>
       <c r="Q15" s="42" t="n"/>
@@ -5480,10 +5482,12 @@
       </c>
       <c r="P21" s="15" t="inlineStr">
         <is>
-          <t>Unanimous segment</t>
-        </is>
-      </c>
-      <c r="Q21" s="42" t="n"/>
+          <t>Language model</t>
+        </is>
+      </c>
+      <c r="Q21" s="42" t="n">
+        <v>0.95</v>
+      </c>
       <c r="R21" s="43" t="n">
         <v>52000</v>
       </c>
@@ -6012,10 +6016,12 @@
       </c>
       <c r="P25" s="15" t="inlineStr">
         <is>
-          <t>Unanimous segment</t>
-        </is>
-      </c>
-      <c r="Q25" s="42" t="n"/>
+          <t>Language model</t>
+        </is>
+      </c>
+      <c r="Q25" s="42" t="n">
+        <v>0.9399999999999999</v>
+      </c>
       <c r="R25" s="43" t="n">
         <v>167000</v>
       </c>

</xml_diff>